<commit_message>
Finalize worker validation and disable Dependabot PRs
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
@@ -1528,7 +1528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1654,6 +1654,11 @@
           <t>description</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>execution_mode</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1750,6 +1755,11 @@
       <c r="T2" s="3" t="inlineStr">
         <is>
           <t>每日2点导入客户文件</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>FULL</t>
         </is>
       </c>
     </row>
@@ -1838,6 +1848,11 @@
           <t>手动触发零售报表导出</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1928,6 +1943,11 @@
           <t>每5分钟分发订单</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2010,6 +2030,11 @@
           <t>每日22点结算</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2106,6 +2131,11 @@
       <c r="T6" t="inlineStr">
         <is>
           <t>FEEDBACK 全链覆盖样本</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>FULL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[codex] centralize env constants and verification scripts (#435)
* fix tenant package excel job config

* Finalize worker validation and disable Dependabot PRs

* chore: separate sql config from shell scripts

* test(worker): extend business scenario matrix

* fix(load): shorten process benchmark account ids

* chore: centralize environment constants and validation scripts

* docs: update preprod pressure verification status

---------

Co-authored-by: idengzhao <40328852+idengzhao@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
@@ -1528,7 +1528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1654,6 +1654,11 @@
           <t>description</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>execution_mode</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1750,6 +1755,11 @@
       <c r="T2" s="3" t="inlineStr">
         <is>
           <t>每日2点导入客户文件</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>FULL</t>
         </is>
       </c>
     </row>
@@ -1838,6 +1848,11 @@
           <t>手动触发零售报表导出</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1928,6 +1943,11 @@
           <t>每5分钟分发订单</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2010,6 +2030,11 @@
           <t>每日22点结算</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2106,6 +2131,11 @@
       <c r="T6" t="inlineStr">
         <is>
           <t>FEEDBACK 全链覆盖样本</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>FULL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(test): tenant-config-package fixtures 补 job_definition.watermark_field 列
console tenant-package import 要求 job_definition sheet 含 watermark_field 表头(schema 加的列),
3 个 fixture 陈旧缺该列 → upload 报 INVALID_ARGUMENT。补空列(nullable)。普通 PG 同样需要,双栈修。

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
@@ -1528,7 +1528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1657,6 +1657,11 @@
       <c r="U1" t="inlineStr">
         <is>
           <t>execution_mode</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>watermark_field</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(routing): biz 多分片路由 CI 集成测试 + 开关文档 + sim reproducible 修复
- BusinessMultiShardRoutingIntegrationTest:把原 env-gated 活体测试转成 CI 可跑——
  起两个真实 PG testcontainer 作 shard-0/shard-1,验 BusinessRoutingDataSourceFactory.multiShard +
  HashAndSiloPlacementResolver(config 路由)/ DbTablePlacementResolver(表覆盖)在真实跨实例下
  把租户连接物理路由到选定片(经 biz.__shard_identity 识别落片)。本地 2/2 绿(~10s)。
- docs/runbook/feature-switches.md:补 batch.datasource.business.routing.* 开关表 + §3.8 说明
  (默认 enabled=false 单片无损;placement-source CONFIG/TABLE;fail-open 语义)。
- scripts/sim/10-process-stage4.sh:seed 改 -f /dev/stdin < file(可重复执行,对齐 #479 范式)。
- test-full-coverage-import-suite/*.xlsx:导入测试数据包更新。

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
@@ -1528,7 +1528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1657,6 +1657,11 @@
       <c r="U1" t="inlineStr">
         <is>
           <t>execution_mode</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>watermark_field</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(routing): biz 多分片路由 CI 集成测试 + 开关文档 + sim reproducible 修复 (#490)
- BusinessMultiShardRoutingIntegrationTest:把原 env-gated 活体测试转成 CI 可跑——
  起两个真实 PG testcontainer 作 shard-0/shard-1,验 BusinessRoutingDataSourceFactory.multiShard +
  HashAndSiloPlacementResolver(config 路由)/ DbTablePlacementResolver(表覆盖)在真实跨实例下
  把租户连接物理路由到选定片(经 biz.__shard_identity 识别落片)。本地 2/2 绿(~10s)。
- docs/runbook/feature-switches.md:补 batch.datasource.business.routing.* 开关表 + §3.8 说明
  (默认 enabled=false 单片无损;placement-source CONFIG/TABLE;fail-open 语义)。
- scripts/sim/10-process-stage4.sh:seed 改 -f /dev/stdin < file(可重复执行,对齐 #479 范式)。
- test-full-coverage-import-suite/*.xlsx:导入测试数据包更新。

Co-authored-by: idengzhao <40328852+idengzhao@users.noreply.github.com>
Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
@@ -1528,7 +1528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1657,6 +1657,11 @@
       <c r="U1" t="inlineStr">
         <is>
           <t>execution_mode</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>watermark_field</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: stabilize sim runtime and graceful shutdown
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
@@ -2748,7 +2748,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>[{"field":"id","rule":"required"}]</t>
+          <t>{"fieldRules":{"customer_no":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_name":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_type":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"status":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"}}}</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>SELECT id, tenant_id, customer_no, customer_name, customer_type, certificate_no, mobile_no, email, status FROM biz.customer_account WHERE tenant_id = :tenantId AND (:batchNo IS NULL OR :batchNo IS NOT NULL)</t>
+          <t>SELECT id, tenant_id, customer_no, customer_name, customer_type, certificate_no, mobile_no, email, status FROM biz.customer_account WHERE tenant_id = :tenantId AND CAST(:batchNo AS text) IS NOT NULL</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -3430,7 +3430,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>[{"field":"id","rule":"required"}]</t>
+          <t>{"fieldRules":{"customer_no":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_name":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_type":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"status":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"}}}</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">

</xml_diff>

<commit_message>
fix: stabilize sim runtime and graceful shutdown (#877)
* fix: stabilize sim runtime and graceful shutdown

* fix: keep quartz restartable during context lifecycle

---------

Co-authored-by: Dengchao <tfys9544@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/ta-tenant-config-package-test.xlsx
@@ -2748,7 +2748,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>[{"field":"id","rule":"required"}]</t>
+          <t>{"fieldRules":{"customer_no":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_name":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_type":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"status":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"}}}</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>SELECT id, tenant_id, customer_no, customer_name, customer_type, certificate_no, mobile_no, email, status FROM biz.customer_account WHERE tenant_id = :tenantId AND (:batchNo IS NULL OR :batchNo IS NOT NULL)</t>
+          <t>SELECT id, tenant_id, customer_no, customer_name, customer_type, certificate_no, mobile_no, email, status FROM biz.customer_account WHERE tenant_id = :tenantId AND CAST(:batchNo AS text) IS NOT NULL</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -3430,7 +3430,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>[{"field":"id","rule":"required"}]</t>
+          <t>{"fieldRules":{"customer_no":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_name":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_type":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"status":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"}}}</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">

</xml_diff>